<commit_message>
changed field names in Excel and query
</commit_message>
<xml_diff>
--- a/api/templates/mtb_detected_rr_detected/mw/en.xlsx
+++ b/api/templates/mtb_detected_rr_detected/mw/en.xlsx
@@ -136,13 +136,13 @@
     <t>Received by</t>
   </si>
   <si>
-    <t>&lt;sampleCollectedOn&gt;</t>
-  </si>
-  <si>
-    <t>&lt;resultWorkflowLogCreatedOn&gt;</t>
-  </si>
-  <si>
-    <t>&lt;resultWorkflowLogOperator&gt;</t>
+    <t>&lt;dateOfSampleCollection&gt;</t>
+  </si>
+  <si>
+    <t>&lt;dateOfReceiptInTheLab&gt;</t>
+  </si>
+  <si>
+    <t>&lt;receivedBy&gt;</t>
   </si>
 </sst>
 </file>

</xml_diff>